<commit_message>
Studio Danielle et la campagne En Mode Actif, cofinancee par l UE
33 nouvelles preuves fortes hors des 271 deja jugees. Classeur A_VERIFIER_2
avec les descriptions completes et une colonne indiquant si la regle D retient
le candidat : elle n en garde que 5 sur 33.

Studio Danielle, 1,74 M d abonnes, quatre videos avec mentions explicites :
en partenariat avec Les Produits Laitiers et leur campagne En Mode Actif
cofinancee par l UE. Le libelle le plus explicite rencontre depuis le debut.

En Mode Actif est ajoutee a la feuille Alias, statut CONFIRME, source primaire.
Elle etait inconnue de la table. Son cofinancement europeen relie au dossier
AGRIP inscrit depuis la premiere session.

Lecon : la troncature des descriptions a 900 caracteres coutait des
decouvertes, pas seulement de la lisibilite.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DfPtphAAkK24cZ5SByH1EW
</commit_message>
<xml_diff>
--- a/cartographie/cartographie_filiere.xlsx
+++ b/cartographie/cartographie_filiere.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Interprofessions'!$A$1:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Industriels'!$A$1:$G$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Marques'!$A$1:$E$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alias'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alias'!$A$1:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Agences'!$A$1:$F$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Influenceurs'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sources_de_donnees'!$A$1:$F$15</definedName>
@@ -12736,7 +12736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12951,32 +12951,36 @@
       <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Le Porc Francais</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>marque filiere</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>INAPORC</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>A VERIFIER</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>En Mode Actif</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>nom de campagne</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRME</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Campagne COFINANCEE PAR L'UNION EUROPEENNE, contre la sedentarite. Nommee par Studio Danielle (1,74 M d'abonnes) dans deux descriptions : « en partenariat avec Les Produits Laitiers et leur campagne En Mode Actif cofinancee par l'UE ». Decouverte le 26/08/2026, absente de la table jusque-la. Le cofinancement europeen relie au dossier AGRIP.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Volaille Francaise</t>
+          <t>Le Porc Francais</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -12986,7 +12990,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>ANVOL</t>
+          <t>INAPORC</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -12999,82 +13003,105 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Volaille Francaise</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>marque filiere</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>ANVOL</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>A VERIFIER</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Oeufs de France</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>marque filiere</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>CNPO</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>A VERIFIER</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>@lescereales</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>compte vitrine</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Intercereales</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>CONFIRME</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>HORS PERIMETRE. Groupe temoin pour tester la detection.</t>
-        </is>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>@lescereales</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>compte vitrine</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Intercereales</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRME</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>HORS PERIMETRE. Groupe temoin pour tester la detection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>@cetepimepate</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>compte vitrine</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>FNPSMS</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>CONFIRME</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>HORS PERIMETRE. Groupe temoin.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>